<commit_message>
Let the emission-factors spreadsheet drive emission-factors.js
Adds scripts/sync-emission-factors.js (npm run sync:factors), which reads
emission-factors-reference.xlsx and rewrites only the changed numbers in
emission-factors.js to match. Reuses the vendored SheetJS build the app
already uses for its own Excel export - no new dependency.

The spreadsheet gains a "JS Path" column (locked) mapping each row to its
exact spot in emission-factors.js, and the Value column is the only
unlocked/editable cell. The sync refuses to write anything if a row has a
non-numeric value or an unrecognized JS Path, and only touches lines whose
value actually changed so it doesn't reformat untouched numbers.

Workflow: edit a Value cell, save, run `npm run sync:factors`, reload.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014YJAb3vBd6Un5zKFTJYt4R
</commit_message>
<xml_diff>
--- a/emission-factors-reference.xlsx
+++ b/emission-factors-reference.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,12 +55,22 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="00555555"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -79,8 +89,20 @@
         <bgColor rgb="00DCE9E3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFEFEF"/>
+        <bgColor rgb="00EFEFEF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -102,11 +124,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -120,13 +186,22 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,14 +567,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,10 +585,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mirrors emission-factors.js at the repo root. This sheet is a read-only reference for reviewing the numbers — to change what the app calculates, edit emission-factors.js directly and this sheet will go stale until manually updated.</t>
+          <t>Edit only the yellow Value cells, save, then run “npm run sync:factors” from the project folder — it rewrites emission-factors.js to match. Don't edit the grey JS Path column; the sync script uses it to find the right spot in the code. Rows with no JS Path are informational only and can't be synced this way.</t>
         </is>
       </c>
     </row>
@@ -539,6 +615,11 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>JS Path</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -549,10 +630,11 @@
           <t>Transport — kg CO2e per passenger-km</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
+      <c r="B5" s="12" t="n"/>
+      <c r="C5" s="12" t="n"/>
+      <c r="D5" s="12" t="n"/>
+      <c r="E5" s="12" t="n"/>
+      <c r="F5" s="13" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -565,7 +647,7 @@
           <t>None / didn't travel</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -573,7 +655,12 @@
           <t>kg CO2e/km</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>TRANSPORT_FACTORS.none</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -586,7 +673,7 @@
           <t>Walk</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -594,7 +681,12 @@
           <t>kg CO2e/km</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>TRANSPORT_FACTORS.walk</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -607,7 +699,7 @@
           <t>Cycle</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -615,7 +707,12 @@
           <t>kg CO2e/km</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>TRANSPORT_FACTORS.cycle</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -628,7 +725,7 @@
           <t>Train</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <v>0.041</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -636,7 +733,12 @@
           <t>kg CO2e/km</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>TRANSPORT_FACTORS.train</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Rough average emission factor.</t>
         </is>
@@ -653,7 +755,7 @@
           <t>Car (blended average)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="7" t="n">
         <v>0.171</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -661,7 +763,12 @@
           <t>kg CO2e/km</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>TRANSPORT_FACTORS.car</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Used whenever the optional car fuel type isn't answered.</t>
         </is>
@@ -673,10 +780,11 @@
           <t>Car fuel type — kg CO2e per km (optional, overrides blended car average)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="13" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -689,7 +797,7 @@
           <t>Diesel</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="7" t="n">
         <v>0.171</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -697,7 +805,12 @@
           <t>kg CO2e/km</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>CAR_FUEL_FACTORS.diesel</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Rough DEFRA-style figure, close to the blended average.</t>
         </is>
@@ -714,7 +827,7 @@
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="7" t="n">
         <v>0.111</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -722,7 +835,12 @@
           <t>kg CO2e/km</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>CAR_FUEL_FACTORS.hybrid</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -735,7 +853,7 @@
           <t>Electric</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="7" t="n">
         <v>0.058</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -743,7 +861,12 @@
           <t>kg CO2e/km</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>CAR_FUEL_FACTORS.electric</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>Uses average UK grid intensity to charge, not tailpipe emissions (there are none).</t>
         </is>
@@ -755,10 +878,11 @@
           <t>Food — meat/fish, kg CO2e per kg of product</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -771,7 +895,7 @@
           <t>Chicken / poultry</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="7" t="n">
         <v>6</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -779,7 +903,12 @@
           <t>kg CO2e/kg</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>MEAT_FACTORS.chicken</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -792,7 +921,7 @@
           <t>Fish / seafood</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="7" t="n">
         <v>5</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -800,7 +929,12 @@
           <t>kg CO2e/kg</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>MEAT_FACTORS.fish</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -813,7 +947,7 @@
           <t>Pork</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="7" t="n">
         <v>7</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -821,7 +955,12 @@
           <t>kg CO2e/kg</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr"/>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>MEAT_FACTORS.pork</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -834,7 +973,7 @@
           <t>Beef</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="7" t="n">
         <v>36</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -842,7 +981,12 @@
           <t>kg CO2e/kg</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>MEAT_FACTORS.beef</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>Roughly 4-6x chicken per commonly cited figures.</t>
         </is>
@@ -859,7 +1003,7 @@
           <t>Lamb</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="7" t="n">
         <v>25</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -867,7 +1011,12 @@
           <t>kg CO2e/kg</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr"/>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>MEAT_FACTORS.lamb</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -880,7 +1029,7 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="7" t="n">
         <v>10</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -888,7 +1037,12 @@
           <t>kg CO2e/kg</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr"/>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>MEAT_FACTORS.other</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -896,10 +1050,11 @@
           <t>Food — portion size, kg of product</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
+      <c r="B22" s="12" t="n"/>
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="13" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -912,7 +1067,7 @@
           <t>Small (~100g)</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="7" t="n">
         <v>0.1</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -920,7 +1075,12 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr"/>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>PORTION_KG.small</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -933,7 +1093,7 @@
           <t>Medium (~150g)</t>
         </is>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="7" t="n">
         <v>0.15</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -941,7 +1101,12 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr"/>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>PORTION_KG.medium</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -954,7 +1119,7 @@
           <t>Large (~250g+)</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n">
+      <c r="C25" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -962,7 +1127,12 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr"/>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>PORTION_KG.large</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -970,10 +1140,11 @@
           <t>Food — per day, kg CO2e per person per day</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
+      <c r="B26" s="12" t="n"/>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="13" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -986,7 +1157,7 @@
           <t>Vegetarian day</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C27" s="7" t="n">
         <v>2.6</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -994,7 +1165,12 @@
           <t>kg CO2e/day</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>FOOD_DAY_FACTORS.veggie</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Rosi et al. 2017 (seven-day diets, ~150 people, Italy).</t>
         </is>
@@ -1011,7 +1187,7 @@
           <t>Vegan day</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C28" s="7" t="n">
         <v>2.3</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1019,7 +1195,12 @@
           <t>kg CO2e/day</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>FOOD_DAY_FACTORS.vegan</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Rosi et al. 2017 (seven-day diets, ~150 people, Italy).</t>
         </is>
@@ -1036,7 +1217,7 @@
           <t>Meat day — non-meat baseline</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C29" s="7" t="n">
         <v>2.6</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1044,9 +1225,10 @@
           <t>kg CO2e/day</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>The rest of a meat day's food (breakfast, sides, etc.) is valued the same as a vegetarian day — the meat is added on top. Always equal to the vegetarian-day figure above.</t>
+      <c r="E29" s="8" t="inlineStr"/>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Not directly editable here — always mirrors the Vegetarian day figure above in emission-factors.js (MEAT_SIDES_BASELINE = FOOD_DAY_FACTORS.veggie), since the rest of a meat day's food isn't any more carbon-efficient than a veggie day. Change the Vegetarian day row instead.</t>
         </is>
       </c>
     </row>
@@ -1056,10 +1238,11 @@
           <t>Food — modelling multipliers</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n"/>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="5" t="n"/>
-      <c r="E30" s="5" t="n"/>
+      <c r="B30" s="12" t="n"/>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="13" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1072,7 +1255,7 @@
           <t>Eating out (dinner only)</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C31" s="7" t="n">
         <v>1.5</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1080,7 +1263,12 @@
           <t>multiplier</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>EATING_OUT_MULTIPLIER</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>Applied to just the dinner slice of a day's food footprint — extra energy use, larger portions, and food waste vs. cooking at home.</t>
         </is>
@@ -1097,7 +1285,7 @@
           <t>Veggie/vegan day dinner share</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n">
+      <c r="C32" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -1105,7 +1293,12 @@
           <t>fraction of day</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>VEGGIE_DINNER_SHARE</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>On a meat day, 'dinner' is the meat portion itself. On a veggie/vegan day there's no such split, so half the flat day figure stands in for dinner.</t>
         </is>
@@ -1117,10 +1310,11 @@
           <t>Food waste — multiplier on food footprint, by self-reported bracket</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
+      <c r="B33" s="12" t="n"/>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="13" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -1133,7 +1327,7 @@
           <t>Low (0-3%)</t>
         </is>
       </c>
-      <c r="C34" s="6" t="n">
+      <c r="C34" s="7" t="n">
         <v>1.02</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -1141,7 +1335,12 @@
           <t>multiplier</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>FOOD_WASTE_MULTIPLIERS.low</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Midpoint of each bracket, applied as 1/(1-waste%): you have to buy/produce more than you actually eat.</t>
         </is>
@@ -1158,7 +1357,7 @@
           <t>Some (3-10%)</t>
         </is>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="C35" s="7" t="n">
         <v>1.07</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -1166,7 +1365,12 @@
           <t>multiplier</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr"/>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>FOOD_WASTE_MULTIPLIERS.some</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1179,7 +1383,7 @@
           <t>High (10-25%)</t>
         </is>
       </c>
-      <c r="C36" s="6" t="n">
+      <c r="C36" s="7" t="n">
         <v>1.25</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -1187,7 +1391,12 @@
           <t>multiplier</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr"/>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>FOOD_WASTE_MULTIPLIERS.high</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -1200,7 +1409,7 @@
           <t>Severe (25%+)</t>
         </is>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="C37" s="7" t="n">
         <v>1.67</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -1208,7 +1417,12 @@
           <t>multiplier</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr"/>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>FOOD_WASTE_MULTIPLIERS.severe</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -1216,10 +1430,11 @@
           <t>Alcohol — kg CO2e per drink</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n"/>
-      <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="5" t="n"/>
+      <c r="B38" s="12" t="n"/>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="13" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -1232,7 +1447,7 @@
           <t>Beer (per pint/can)</t>
         </is>
       </c>
-      <c r="C39" s="6" t="n">
+      <c r="C39" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -1240,7 +1455,12 @@
           <t>kg CO2e/drink</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>BEER_KG_PER_DRINK</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>Covers production, packaging, and transport.</t>
         </is>
@@ -1257,7 +1477,7 @@
           <t>Wine (per ~175ml glass)</t>
         </is>
       </c>
-      <c r="C40" s="6" t="n">
+      <c r="C40" s="7" t="n">
         <v>0.3</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -1265,7 +1485,12 @@
           <t>kg CO2e/glass</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr"/>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>WINE_KG_PER_GLASS</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -1278,7 +1503,7 @@
           <t>Spirits (per 25ml shot @ 40% ABV)</t>
         </is>
       </c>
-      <c r="C41" s="6" t="n">
+      <c r="C41" s="7" t="n">
         <v>0.15</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -1286,7 +1511,12 @@
           <t>kg CO2e/shot</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>SPIRITS_KG_PER_SHOT_AT_40PCT</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>Scales linearly with actual ABV entered.</t>
         </is>
@@ -1298,10 +1528,11 @@
           <t>Flights — kg CO2e per return flight</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="5" t="n"/>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="5" t="n"/>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="13" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -1314,7 +1545,7 @@
           <t>Short-haul (European)</t>
         </is>
       </c>
-      <c r="C43" s="6" t="n">
+      <c r="C43" s="7" t="n">
         <v>250</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -1322,7 +1553,12 @@
           <t>kg CO2e/flight</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr"/>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>SHORT_HAUL_FLIGHT_KG</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -1335,7 +1571,7 @@
           <t>Long-haul (international)</t>
         </is>
       </c>
-      <c r="C44" s="6" t="n">
+      <c r="C44" s="7" t="n">
         <v>1600</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -1343,7 +1579,12 @@
           <t>kg CO2e/flight</t>
         </is>
       </c>
-      <c r="E44" s="7" t="inlineStr"/>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>LONG_HAUL_FLIGHT_KG</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -1351,10 +1592,11 @@
           <t>Home energy</t>
         </is>
       </c>
-      <c r="B45" s="5" t="n"/>
-      <c r="C45" s="5" t="n"/>
-      <c r="D45" s="5" t="n"/>
-      <c r="E45" s="5" t="n"/>
+      <c r="B45" s="12" t="n"/>
+      <c r="C45" s="12" t="n"/>
+      <c r="D45" s="12" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="13" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -1367,7 +1609,7 @@
           <t>Grid electricity</t>
         </is>
       </c>
-      <c r="C46" s="6" t="n">
+      <c r="C46" s="7" t="n">
         <v>0.2</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -1375,7 +1617,12 @@
           <t>kg CO2e/kWh</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>GRID_ELECTRICITY_KG_PER_KWH</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
         <is>
           <t>Rough average grid electricity factor.</t>
         </is>
@@ -1392,7 +1639,7 @@
           <t>Gas/oil heating</t>
         </is>
       </c>
-      <c r="C47" s="6" t="n">
+      <c r="C47" s="7" t="n">
         <v>0.18</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -1400,7 +1647,12 @@
           <t>kg CO2e/kWh</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>GAS_HEATING_KG_PER_KWH</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>Rough blended gas/oil heating factor.</t>
         </is>
@@ -1412,10 +1664,11 @@
           <t>Goods &amp; car ownership</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n"/>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="5" t="n"/>
-      <c r="E48" s="5" t="n"/>
+      <c r="B48" s="12" t="n"/>
+      <c r="C48" s="12" t="n"/>
+      <c r="D48" s="12" t="n"/>
+      <c r="E48" s="12" t="n"/>
+      <c r="F48" s="13" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -1428,7 +1681,7 @@
           <t>Clothing item</t>
         </is>
       </c>
-      <c r="C49" s="6" t="n">
+      <c r="C49" s="7" t="n">
         <v>10</v>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -1436,7 +1689,12 @@
           <t>kg CO2e/item</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>CLOTHING_ITEM_KG</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
         <is>
           <t>Rough blended average per clothing item.</t>
         </is>
@@ -1453,7 +1711,7 @@
           <t>Manufacturing (amortized)</t>
         </is>
       </c>
-      <c r="C50" s="6" t="n">
+      <c r="C50" s="7" t="n">
         <v>700</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -1461,7 +1719,12 @@
           <t>kg CO2e/year</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr">
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>CAR_MANUFACTURING_AMORTIZED_KG_PER_YEAR</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
         <is>
           <t>Rough embodied build footprint, amortized over an ~14yr average car lifetime.</t>
         </is>
@@ -1473,10 +1736,11 @@
           <t>Pets — kg CO2e per year</t>
         </is>
       </c>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="5" t="n"/>
+      <c r="B51" s="12" t="n"/>
+      <c r="C51" s="12" t="n"/>
+      <c r="D51" s="12" t="n"/>
+      <c r="E51" s="12" t="n"/>
+      <c r="F51" s="13" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -1489,7 +1753,7 @@
           <t>Dog</t>
         </is>
       </c>
-      <c r="C52" s="6" t="n">
+      <c r="C52" s="7" t="n">
         <v>770</v>
       </c>
       <c r="D52" s="6" t="inlineStr">
@@ -1497,7 +1761,12 @@
           <t>kg CO2e/year</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr">
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>DOG_KG_PER_YEAR</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
         <is>
           <t>Mostly diet-driven.</t>
         </is>
@@ -1514,7 +1783,7 @@
           <t>Cat</t>
         </is>
       </c>
-      <c r="C53" s="6" t="n">
+      <c r="C53" s="7" t="n">
         <v>310</v>
       </c>
       <c r="D53" s="6" t="inlineStr">
@@ -1522,7 +1791,12 @@
           <t>kg CO2e/year</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr"/>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>CAT_KG_PER_YEAR</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -1530,10 +1804,11 @@
           <t>Water</t>
         </is>
       </c>
-      <c r="B54" s="5" t="n"/>
-      <c r="C54" s="5" t="n"/>
-      <c r="D54" s="5" t="n"/>
-      <c r="E54" s="5" t="n"/>
+      <c r="B54" s="12" t="n"/>
+      <c r="C54" s="12" t="n"/>
+      <c r="D54" s="12" t="n"/>
+      <c r="E54" s="12" t="n"/>
+      <c r="F54" s="13" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -1546,7 +1821,7 @@
           <t>Mains water (supply + treatment)</t>
         </is>
       </c>
-      <c r="C55" s="6" t="n">
+      <c r="C55" s="7" t="n">
         <v>0.32</v>
       </c>
       <c r="D55" s="6" t="inlineStr">
@@ -1554,7 +1829,12 @@
           <t>kg CO2e/m3</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>WATER_KG_PER_M3</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
         <is>
           <t>Rough DEFRA-style combined factor.</t>
         </is>
@@ -1566,10 +1846,11 @@
           <t>Banking — kg CO2e financed per £1 held per year</t>
         </is>
       </c>
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="5" t="n"/>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="5" t="n"/>
+      <c r="B56" s="12" t="n"/>
+      <c r="C56" s="12" t="n"/>
+      <c r="D56" s="12" t="n"/>
+      <c r="E56" s="12" t="n"/>
+      <c r="F56" s="13" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -1582,7 +1863,7 @@
           <t>Barclays</t>
         </is>
       </c>
-      <c r="C57" s="6" t="n">
+      <c r="C57" s="7" t="n">
         <v>0.2376</v>
       </c>
       <c r="D57" s="6" t="inlineStr">
@@ -1590,7 +1871,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr"/>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.barclays</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -1603,7 +1889,7 @@
           <t>HSBC</t>
         </is>
       </c>
-      <c r="C58" s="6" t="n">
+      <c r="C58" s="7" t="n">
         <v>0.217</v>
       </c>
       <c r="D58" s="6" t="inlineStr">
@@ -1611,7 +1897,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E58" s="7" t="inlineStr"/>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.hsbc</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -1624,7 +1915,7 @@
           <t>First Direct</t>
         </is>
       </c>
-      <c r="C59" s="6" t="n">
+      <c r="C59" s="7" t="n">
         <v>0.217</v>
       </c>
       <c r="D59" s="6" t="inlineStr">
@@ -1632,7 +1923,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr"/>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.firstDirect</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -1645,7 +1941,7 @@
           <t>Chase</t>
         </is>
       </c>
-      <c r="C60" s="6" t="n">
+      <c r="C60" s="7" t="n">
         <v>0.1897</v>
       </c>
       <c r="D60" s="6" t="inlineStr">
@@ -1653,7 +1949,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E60" s="7" t="inlineStr"/>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.chase</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -1666,7 +1967,7 @@
           <t>Santander</t>
         </is>
       </c>
-      <c r="C61" s="6" t="n">
+      <c r="C61" s="7" t="n">
         <v>0.1742</v>
       </c>
       <c r="D61" s="6" t="inlineStr">
@@ -1674,7 +1975,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr"/>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.santander</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -1687,7 +1993,7 @@
           <t>NatWest</t>
         </is>
       </c>
-      <c r="C62" s="6" t="n">
+      <c r="C62" s="7" t="n">
         <v>0.1295</v>
       </c>
       <c r="D62" s="6" t="inlineStr">
@@ -1695,7 +2001,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E62" s="7" t="inlineStr"/>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.natwest</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -1708,7 +2019,7 @@
           <t>RBS</t>
         </is>
       </c>
-      <c r="C63" s="6" t="n">
+      <c r="C63" s="7" t="n">
         <v>0.1295</v>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -1716,7 +2027,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E63" s="7" t="inlineStr"/>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.rbs</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -1729,7 +2045,7 @@
           <t>Monzo</t>
         </is>
       </c>
-      <c r="C64" s="6" t="n">
+      <c r="C64" s="7" t="n">
         <v>0.1088</v>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -1737,7 +2053,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr"/>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.monzo</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -1750,7 +2071,7 @@
           <t>Lloyds</t>
         </is>
       </c>
-      <c r="C65" s="6" t="n">
+      <c r="C65" s="7" t="n">
         <v>0.0704</v>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -1758,7 +2079,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E65" s="7" t="inlineStr"/>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.lloyds</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
@@ -1771,7 +2097,7 @@
           <t>Halifax</t>
         </is>
       </c>
-      <c r="C66" s="6" t="n">
+      <c r="C66" s="7" t="n">
         <v>0.0704</v>
       </c>
       <c r="D66" s="6" t="inlineStr">
@@ -1779,7 +2105,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E66" s="7" t="inlineStr"/>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.halifax</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -1792,7 +2123,7 @@
           <t>Metro Bank</t>
         </is>
       </c>
-      <c r="C67" s="6" t="n">
+      <c r="C67" s="7" t="n">
         <v>0.0694</v>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -1800,7 +2131,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E67" s="7" t="inlineStr"/>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.metroBank</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -1813,7 +2149,7 @@
           <t>Starling</t>
         </is>
       </c>
-      <c r="C68" s="6" t="n">
+      <c r="C68" s="7" t="n">
         <v>0.061</v>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -1821,7 +2157,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E68" s="7" t="inlineStr"/>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.starling</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -1834,7 +2175,7 @@
           <t>Virgin Money</t>
         </is>
       </c>
-      <c r="C69" s="6" t="n">
+      <c r="C69" s="7" t="n">
         <v>0.0517</v>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -1842,7 +2183,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E69" s="7" t="inlineStr"/>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.virginMoney</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
@@ -1855,7 +2201,7 @@
           <t>Nationwide</t>
         </is>
       </c>
-      <c r="C70" s="6" t="n">
+      <c r="C70" s="7" t="n">
         <v>0.0432</v>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -1863,7 +2209,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E70" s="7" t="inlineStr"/>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.nationwide</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -1876,7 +2227,7 @@
           <t>The Co-operative Bank</t>
         </is>
       </c>
-      <c r="C71" s="6" t="n">
+      <c r="C71" s="7" t="n">
         <v>0.0328</v>
       </c>
       <c r="D71" s="6" t="inlineStr">
@@ -1884,7 +2235,12 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr"/>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.cooperative</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -1897,7 +2253,7 @@
           <t>Triodos</t>
         </is>
       </c>
-      <c r="C72" s="6" t="n">
+      <c r="C72" s="7" t="n">
         <v>0.0317</v>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -1905,15 +2261,20 @@
           <t>kg CO2e/£/year</t>
         </is>
       </c>
-      <c r="E72" s="7" t="inlineStr"/>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>BANK_KG_PER_POUND_PER_YEAR.triodos</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="inlineStr">
+      <c r="A73" s="10" t="inlineStr">
         <is>
           <t>Banking</t>
         </is>
       </c>
-      <c r="B73" s="9" t="inlineStr">
+      <c r="B73" s="11" t="inlineStr">
         <is>
           <t>Source: MotherTree bank carbon emissions league table — tCO2 financed per £10,000 held, reflecting each bank's fossil-fuel financing intensity (mymothertree.com/bank-league-table). tCO2/£10k x 0.1 = kg/£.</t>
         </is>
@@ -1925,10 +2286,11 @@
           <t>Reference — for comparisons</t>
         </is>
       </c>
-      <c r="B74" s="5" t="n"/>
-      <c r="C74" s="5" t="n"/>
-      <c r="D74" s="5" t="n"/>
-      <c r="E74" s="5" t="n"/>
+      <c r="B74" s="12" t="n"/>
+      <c r="C74" s="12" t="n"/>
+      <c r="D74" s="12" t="n"/>
+      <c r="E74" s="12" t="n"/>
+      <c r="F74" s="13" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -1941,7 +2303,7 @@
           <t>Mature tree, CO2 absorbed</t>
         </is>
       </c>
-      <c r="C75" s="6" t="n">
+      <c r="C75" s="7" t="n">
         <v>22</v>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -1949,32 +2311,38 @@
           <t>kg CO2/year</t>
         </is>
       </c>
-      <c r="E75" s="7" t="inlineStr">
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>TREE_KG_PER_YEAR</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="inlineStr">
         <is>
           <t>Rough figure for one mature tree per year.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="18">
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A74:E74"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="B73:F73"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>